<commit_message>
Add new PDF files on Datenschutz, Deepfakes, Halluzinationen, and Prompting techniques. These documents cover essential topics such as data privacy in AI, recognizing and responding to deepfakes, understanding AI hallucinations, and effective prompting strategies for better AI interactions.
</commit_message>
<xml_diff>
--- a/data/Copilot_Beispiel.xlsx
+++ b/data/Copilot_Beispiel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gollnickdatasolutions-my.sharepoint.com/personal/bertgollnick_gollnickdatasolutions_onmicrosoft_com/Documents/Projects/Bildungsurlaub/KIfürJobUndAlltag/Inhalte/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{8FA7408D-3C2B-4F53-A247-F32E65FC1004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F7C8656-644F-4DB3-AA2A-9A5782295704}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{8FA7408D-3C2B-4F53-A247-F32E65FC1004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F03B5633-C749-4378-9F07-40BF552FE44E}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{9FC30950-8112-467D-B040-64EA03D87939}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9FC30950-8112-467D-B040-64EA03D87939}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Ich habe einhundert € für das Abo bezahlt.</t>
   </si>
@@ -67,9 +67,6 @@
   </si>
   <si>
     <t>Netflix kostet mittlerweile zehn Euronen im Monat.</t>
-  </si>
-  <si>
-    <t>franziska.rueckert@drv-bund.de; Markus Güntther &lt;markus.guenther.inbox@outlook.de&gt;; Matthias Täubrich &lt;matthias@taeubrich.de&gt;; blauth.timo@yahoo.de; sarah.roesener@web.de; Jesko Rehberg &lt;jesko.rehberg@dar-analytics.de&gt;; franziskarueckert@gmx.net</t>
   </si>
 </sst>
 </file>
@@ -122,6 +119,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -441,7 +442,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ABA0037-5822-4E2F-98F7-674D229CE257}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="53.5703125" bestFit="1" customWidth="1"/>
@@ -466,11 +467,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>